<commit_message>
feat(hw): VISOR 측위 포드(UWB DWM3000 + GPS) ― 대원 위치를 트윈에
실내(GPS 차폐)에서도 대원 위치가 지휘 트윈에 뜨도록 UWB 정밀측위 추가.
- SCAD: nav_pod() 모듈(헬멧 레일 위 라이저로 물리 접촉, GPS 패치 상단 +
  UWB 모노폴 전방 + fix LED), PART_MODE=NAV_POD. visor.stl 재-export.
- BOM: UWB DWM3000 + UWB 안테나 추가(VISOR 878, 총 4,790).
- 조립가이드: A-7.5 측위 포드 조립 스텝(앵커/폴백 포함).
- 회로설계: UWB SPI0+IRQ+RST / GNSS UART, NAV 포드 8핀 핀아웃, 융합 측위 노트.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaurVEcuaFqxGKrpuZ17se
</commit_message>
<xml_diff>
--- a/hardware/bom/FRIZE_BOM.xlsx
+++ b/hardware/bom/FRIZE_BOM.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONSOLE-1 콘솔" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VISOR-1 고글" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCOUT-1 드론" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VENT-1 IoT포트" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SW-HW 연결" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공구·소모품" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CONSOLE-1 콘솔" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="VISOR-1 고글" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SCOUT-1 드론" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="VENT-1 IoT포트" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SW-HW 연결" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="공구·소모품" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>작성일 2026-06-19 · 단가 추정 USD · 환율 1380 KRW/USD</t>
+          <t>작성일 2026-06-20 · 단가 추정 USD · 환율 1380 KRW/USD</t>
         </is>
       </c>
     </row>
@@ -539,10 +539,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7842</v>
+        <v>7878</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>10821960</v>
+        <v>10871640</v>
       </c>
     </row>
     <row r="7">
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>24754</v>
+        <v>24790</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>34160520</v>
+        <v>34210200</v>
       </c>
     </row>
     <row r="12">
@@ -617,10 +617,10 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>49901</v>
+        <v>50009</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>68863380</v>
+        <v>69012420</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1428,397 +1428,405 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>cm급 위치</t>
+          <t>옥외 cm급 위치</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CO 가스센서</t>
+          <t>UWB 실내측위 모듈</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Alphasense 전기화학식 CO</t>
+          <t>Qorvo DWM3000 (DW3110, 802.15.4z)</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>82800</v>
-      </c>
-      <c r="G12" s="4" t="inlineStr"/>
+        <v>38640</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>★실내 0.1~0.3m 측위(GPS 차폐 보완)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>O2 가스센서</t>
+          <t>UWB 안테나</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>전기화학식 산소 농도</t>
+          <t>UWB 칩 안테나 + 동축</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>110400</v>
+        <v>11040</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>산소결핍 경보</t>
+          <t>nav 포드 모노폴</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>가연성가스(LEL) 센서</t>
+          <t>CO 가스센서</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>촉매연소/NDIR LEL</t>
+          <t>Alphasense 전기화학식 CO</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>165600</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>폭발하한 감지</t>
-        </is>
-      </c>
+        <v>82800</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>H2S/HCN 센서</t>
+          <t>O2 가스센서</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>전기화학식 황화수소/시안화수소</t>
+          <t>전기화학식 산소 농도</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>124200</v>
+        <v>110400</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>유독가스</t>
+          <t>산소결핍 경보</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>온도 측정보드</t>
+          <t>가연성가스(LEL) 센서</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>K타입 열전대 + 주변온도</t>
+          <t>촉매연소/NDIR LEL</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>48300</v>
-      </c>
-      <c r="G16" s="4" t="inlineStr"/>
+        <v>165600</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>폭발하한 감지</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>MEMS 마이크 어레이</t>
+          <t>H2S/HCN 센서</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>3채널 빔포밍</t>
+          <t>전기화학식 황화수소/시안화수소</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>24840</v>
+        <v>124200</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>음성→텍스트</t>
+          <t>유독가스</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>골전도 트랜스듀서</t>
+          <t>온도 측정보드</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>양쪽 골전도 스피커</t>
+          <t>K타입 열전대 + 주변온도</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>55200</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>귀 막혀도 들림</t>
-        </is>
-      </c>
+        <v>48300</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>5G 모뎀</t>
+          <t>MEMS 마이크 어레이</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Quectel RM502Q-AE</t>
+          <t>3채널 빔포밍</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>260</v>
+        <v>18</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>260</v>
+        <v>18</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>358800</v>
-      </c>
-      <c r="G19" s="4" t="inlineStr"/>
+        <v>24840</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>음성→텍스트</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>서브기가 메시 라디오</t>
+          <t>골전도 트랜스듀서</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>RFD900x 계열 mesh</t>
+          <t>양쪽 골전도 스피커</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>130</v>
+        <v>40</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>179400</v>
+        <v>55200</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>통신 두절 대비</t>
+          <t>귀 막혀도 들림</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>WiFi6E/BT M.2</t>
+          <t>5G 모뎀</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>근거리 고대역</t>
+          <t>Quectel RM502Q-AE</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>35</v>
+        <v>260</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>35</v>
+        <v>260</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>48300</v>
+        <v>358800</v>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>안테나 세트</t>
+          <t>서브기가 메시 라디오</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>5G/GNSS/메시/WiFi</t>
+          <t>RFD900x 계열 mesh</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>82800</v>
-      </c>
-      <c r="G22" s="4" t="inlineStr"/>
+        <v>179400</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>통신 두절 대비</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>핫스왑 배터리팩</t>
+          <t>WiFi6E/BT M.2</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>21700 듀얼셀 내열팩</t>
+          <t>근거리 고대역</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>240</v>
+        <v>35</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>331200</v>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>현장에서 갈아끼움</t>
-        </is>
-      </c>
+        <v>48300</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>전원관리 보드(PMIC)</t>
+          <t>안테나 세트</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>커스텀 다중레일 PMIC</t>
+          <t>5G/GNSS/메시/WiFi</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>124200</v>
+        <v>82800</v>
       </c>
       <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>냉각 어셈블리</t>
+          <t>핫스왑 배터리팩</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>히트파이프 + 마이크로 블로워(밀폐)</t>
+          <t>21700 듀얼셀 내열팩</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>55</v>
+        <v>240</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>75900</v>
-      </c>
-      <c r="G25" s="4" t="inlineStr"/>
+        <v>331200</v>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>현장에서 갈아끼움</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>AR 커버 렌즈</t>
+          <t>전원관리 보드(PMIC)</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>내열/내스크래치 곡면 커버</t>
+          <t>커스텀 다중레일 PMIC</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
@@ -1838,176 +1846,226 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>외부 하우징</t>
+          <t>냉각 어셈블리</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>CNC 알루미늄 + 세라믹 코팅 (프로토)</t>
+          <t>히트파이프 + 마이크로 블로워(밀폐)</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>250</v>
+        <v>55</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>250</v>
+        <v>55</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>345000</v>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>★타협X</t>
-        </is>
-      </c>
+        <v>75900</v>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>내부 프레임</t>
+          <t>AR 커버 렌즈</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>PC-CF 프린트 부품 일체</t>
+          <t>내열/내스크래치 곡면 커버</t>
         </is>
       </c>
       <c r="C28" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>55200</v>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>scad에서 뽑음</t>
-        </is>
-      </c>
+        <v>124200</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>FFC/FPC 플렉스케이블</t>
+          <t>외부 하우징</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>카메라/디스플레이 배선 세트</t>
+          <t>CNC 알루미늄 + 세라믹 코팅 (프로토)</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>45</v>
+        <v>250</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>45</v>
+        <v>250</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>62100</v>
-      </c>
-      <c r="G29" s="4" t="inlineStr"/>
+        <v>345000</v>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>★타협X</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>체결/커넥터/배선</t>
+          <t>내부 프레임</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>방진방수 커넥터, 하네스</t>
+          <t>PC-CF 프린트 부품 일체</t>
         </is>
       </c>
       <c r="C30" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>96600</v>
-      </c>
-      <c r="G30" s="4" t="inlineStr"/>
+        <v>55200</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>scad에서 뽑음</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>스토리지</t>
+          <t>FFC/FPC 플렉스케이블</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>NVMe 256GB</t>
+          <t>카메라/디스플레이 배선 세트</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>55200</v>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>로그/모델</t>
-        </is>
-      </c>
+        <v>62100</v>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
+          <t>체결/커넥터/배선</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>방진방수 커넥터, 하네스</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>96600</v>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>스토리지</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>NVMe 256GB</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>55200</v>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>로그/모델</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
           <t>헬멧/SCBA 마운트</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>NFPA 헬멧 레일 + 마스크 인터페이스</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="5" t="n">
+      <c r="C34" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="E34" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="F32" s="5" t="n">
+      <c r="F34" s="5" t="n">
         <v>110400</v>
       </c>
-      <c r="G32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="D33" s="10" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>7842</v>
-      </c>
-      <c r="F33" s="11" t="n">
-        <v>10821960</v>
+      <c r="E35" s="11" t="n">
+        <v>7878</v>
+      </c>
+      <c r="F35" s="11" t="n">
+        <v>10871640</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(hw+sw): ANCHOR-1 UWB 비콘 + 드론 디스펜서 + DeployAnchor 명령
드론이 진입 시 UWB 측위 비콘을 '맨 처음' 투하해 실내 측위망을 깐다.
- frize_anchor.scad: 자기복원(무게추) 드롭 비콘 ― 범퍼링+UWB 돔+LED+후크.
- frize_scout_frame.scad: anchor_dispenser() 3발 매거진+서보 게이트(벨리 하부).
- BOM: ANCHOR-1(6발 12) 시트+표+합계, SCOUT 디스펜서 부품. 총 4,875.
- schema: CommandAction::DeployAnchor.
- scout: DeployAnchor → 비콘 투하(매거진 차감) + 위치 Detection 송출(트윈 표시).
STL 재-export, 직렬화 검증 완료.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaurVEcuaFqxGKrpuZ17se
</commit_message>
<xml_diff>
--- a/hardware/bom/FRIZE_BOM.xlsx
+++ b/hardware/bom/FRIZE_BOM.xlsx
@@ -12,8 +12,9 @@
     <sheet name="VISOR-1 고글" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="SCOUT-1 드론" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="VENT-1 IoT포트" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SW-HW 연결" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="공구·소모품" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ANCHOR-1 UWB비콘" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SW-HW 연결" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="공구·소모품" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -552,10 +553,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8908</v>
+        <v>8993</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>12293040</v>
+        <v>12410340</v>
       </c>
     </row>
     <row r="8">
@@ -574,53 +575,66 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>SW↔HW 연결/인터페이스 (1세트)</t>
+          <t>ANCHOR-1 UWB 측위 비콘 (6발 세트)</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>830</v>
+        <v>312</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>1145400</v>
+        <v>430560</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>SW↔HW 연결/인터페이스 (1세트)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>830</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>1145400</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>공구/소모품 (1세트, 1회성)</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B11" s="5" t="n">
         <v>1665</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C11" s="5" t="n">
         <v>2297700</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>── 지휘소 1식 (콘솔+고글+드론+VENT+연결+공구)</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>24790</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>34210200</v>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>참고: 콘솔1+고글3+드론2+VENT2+연결+공구1 운영세트</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>50009</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>69012420</v>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>── 지휘소 1식 (콘솔+고글+드론+VENT+앵커+연결+공구)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>25187</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>34758060</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>참고: 콘솔1+고글3+드론2+VENT2+앵커12+연결+공구1 운영세트</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>50803</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>70108140</v>
       </c>
     </row>
   </sheetData>
@@ -2079,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2779,16 +2793,74 @@
       <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="D29" s="10" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>UWB 앵커 디스펜서</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>3발 매거진 + 서보 게이트(scad DISPENSER)</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>82800</v>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>★진입 시 비콘 투하</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>디스펜서 서보+릴리즈</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>메탈기어 서보 + 게이트 슬라이드</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>34500</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>1발씩 낙하</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>8908</v>
-      </c>
-      <c r="F29" s="11" t="n">
-        <v>12293040</v>
+      <c r="E31" s="11" t="n">
+        <v>8993</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>12410340</v>
       </c>
     </row>
   </sheetData>
@@ -3255,7 +3327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3270,7 +3342,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SW ↔ HW 연결 / 인터페이스 (소프트웨어가 하드웨어를 구동하는 접점)</t>
+          <t>FRIZE ANCHOR-1 ― 드론 투하 UWB 측위 비콘 BOM (6발)</t>
         </is>
       </c>
     </row>
@@ -3321,48 +3393,48 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>센서 통합 MCU 보드</t>
+          <t>UWB 비콘 MCU</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>STM32F4 ― 가스4종/IMU 집약→Jetson(USB-CDC), frize_visor sensors HAL</t>
+          <t>ESP32-C3 + Qorvo DWM3000(앵커 모드)</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>36</v>
+        <v>132</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>49680</v>
+        <v>182160</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>고글+가스포드 펌웨어</t>
+          <t>삼변측량 앵커</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>USB-UART 어댑터</t>
+          <t>UWB 안테나</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>FTDI FT232H ― Pixhawk TELEM2 ↔ Jetson(MAVLink/MAVSDK)</t>
+          <t>칩 안테나 + 매칭</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>24</v>
@@ -3370,293 +3442,131 @@
       <c r="F6" s="5" t="n">
         <v>33120</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>frize_scout flight</t>
-        </is>
-      </c>
+      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>GMSL2 SerDes 보드</t>
+          <t>배터리(단셀)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>열화상/RGB 카메라 장거리 시리얼라이저-디시리얼라이저</t>
+          <t>21700 + 보호회로(저온 대응)</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>120</v>
+        <v>9</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>360</v>
+        <v>54</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>496800</v>
+        <v>74520</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>FLIR/Sony→Jetson CSI</t>
+          <t>수 시간 가동</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>LiDAR 이더넷 어댑터+스위치</t>
+          <t>자기복원 무게추</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Livox Mid-360 기가비트 인터페이스 + 소형 산업 스위치</t>
+          <t>텅스텐/스틸 베이스(굴러서 똑바로)</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>70</v>
+        <v>6</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>96600</v>
+        <v>49680</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>frize_mapping 입력</t>
+          <t>self-righting</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>레벨 시프터/버스 보드</t>
+          <t>충격흡수 범퍼+셸</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>3.3↔5V, I2C/SPI 분기(센서 다중 연결)</t>
+          <t>TPU 범퍼 + 고시인성 PC 셸</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>55200</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr"/>
+        <v>66240</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>scad frize_anchor</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>ST-Link V3 디버거</t>
+          <t>상태 LED/스위치</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>MCU 펌웨어 플래싱/디버그</t>
+          <t>투하·fix 표시, 자동 전원</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>41400</v>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>센서보드 부트로더</t>
-        </is>
-      </c>
+        <v>24840</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>CAN 트랜시버 모듈</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>ESC/배터리 텔레메트리(드론 상태→SW)</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>41400</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>커넥터/시그널 케이블 키트</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>JST-GH, Molex, 실드 신호선(전 모듈 배선)</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>62100</v>
-      </c>
-      <c r="G12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>microSD 128GB(산업용)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Jetson OS/FRIZE 이미지 플래싱</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>82800</v>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>고글2+드론1</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>절연 USB 허브</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>UVC 카메라/주변장치 다중 + 노이즈 절연</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>96600</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>RTC/PPS 시각동기 모듈</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>센서·영상 타임스탬프 정합(융합 정확도)</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>34500</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>frize_mapping 정합</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>PoE 인젝터/DC-DC</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>컴퓨트·LiDAR 안정 급전(전원↔데이터)</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>55200</v>
-      </c>
-      <c r="G16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>830</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>1145400</v>
+      <c r="E11" s="11" t="n">
+        <v>312</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>430560</v>
       </c>
     </row>
   </sheetData>
@@ -3685,6 +3595,421 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>SW ↔ HW 연결 / 인터페이스 (소프트웨어가 하드웨어를 구동하는 접점)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>단가/합계는 추정치(USD). KRW는 환율 1380 적용.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>부품</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>스펙 / 모델</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>단가(USD)</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>소계(USD)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>소계(KRW)</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>센서 통합 MCU 보드</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>STM32F4 ― 가스4종/IMU 집약→Jetson(USB-CDC), frize_visor sensors HAL</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>49680</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>고글+가스포드 펌웨어</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>USB-UART 어댑터</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>FTDI FT232H ― Pixhawk TELEM2 ↔ Jetson(MAVLink/MAVSDK)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>33120</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>frize_scout flight</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GMSL2 SerDes 보드</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>열화상/RGB 카메라 장거리 시리얼라이저-디시리얼라이저</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>496800</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>FLIR/Sony→Jetson CSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>LiDAR 이더넷 어댑터+스위치</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Livox Mid-360 기가비트 인터페이스 + 소형 산업 스위치</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>96600</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>frize_mapping 입력</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>레벨 시프터/버스 보드</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>3.3↔5V, I2C/SPI 분기(센서 다중 연결)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>55200</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>ST-Link V3 디버거</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>MCU 펌웨어 플래싱/디버그</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>41400</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>센서보드 부트로더</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CAN 트랜시버 모듈</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ESC/배터리 텔레메트리(드론 상태→SW)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>41400</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>커넥터/시그널 케이블 키트</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>JST-GH, Molex, 실드 신호선(전 모듈 배선)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>62100</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>microSD 128GB(산업용)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Jetson OS/FRIZE 이미지 플래싱</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>82800</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>고글2+드론1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>절연 USB 허브</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>UVC 카메라/주변장치 다중 + 노이즈 절연</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>96600</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>RTC/PPS 시각동기 모듈</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>센서·영상 타임스탬프 정합(융합 정확도)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>34500</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>frize_mapping 정합</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>PoE 인젝터/DC-DC</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>컴퓨트·LiDAR 안정 급전(전원↔데이터)</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>55200</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>830</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>1145400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>공구 / 소모품 (차고 셋업)</t>
         </is>
       </c>

</xml_diff>